<commit_message>
Versión con mejoraras de UX y correción de errores
</commit_message>
<xml_diff>
--- a/Output/Precio de software TEKNOGADGET.xlsx
+++ b/Output/Precio de software TEKNOGADGET.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario 1\Documents\Proyectos de C#\TecnogadgedWin7\Output\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UZIEL\OneDrive\Documents\FREELANCER\TecnogadgedWin7\Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECA9C22E-0BEA-4A92-B25A-B8423C8FF3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B98FE7-8208-4073-B6BD-00250C83D93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{48C9FD5F-70C1-44D7-83C9-0F804B9CE7E4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{48C9FD5F-70C1-44D7-83C9-0F804B9CE7E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
   <si>
     <t>Modulos</t>
   </si>
@@ -151,6 +151,18 @@
   </si>
   <si>
     <t>Backup de base de datos</t>
+  </si>
+  <si>
+    <t>Implementación de comentarios y refacciones en la tabla y filtrado por fechas (Cambios en la BD)</t>
+  </si>
+  <si>
+    <t>Nuevo diseño de la vista de empleados (Con detalles)</t>
+  </si>
+  <si>
+    <t>Margen de error</t>
+  </si>
+  <si>
+    <t>15/3/2025 pago 700</t>
   </si>
 </sst>
 </file>
@@ -161,7 +173,7 @@
     <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-[$$-80A]* #,##0.00_-;\-[$$-80A]* #,##0.00_-;_-[$$-80A]* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -183,8 +195,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -260,6 +280,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF7C80"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -318,7 +344,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -340,16 +366,25 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="13" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Currency" xfId="1" builtinId="4"/>
+    <cellStyle name="Moneda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFF7C80"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -362,9 +397,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -402,7 +437,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -508,7 +543,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -650,7 +685,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -658,8 +693,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE51DA6-4F34-4E63-B58F-F2E67A00BE67}">
-  <dimension ref="B2:I33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:L33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
     <col min="3" max="3" width="91.140625" customWidth="1"/>
@@ -669,22 +704,22 @@
     <col min="8" max="8" width="12.28515625" customWidth="1"/>
     <col min="9" max="9" width="20.85546875" customWidth="1"/>
     <col min="10" max="10" width="16.85546875" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" customWidth="1"/>
+    <col min="11" max="11" width="23.5703125" customWidth="1"/>
     <col min="12" max="12" width="20.7109375" customWidth="1"/>
     <col min="13" max="13" width="36.28515625" customWidth="1"/>
     <col min="14" max="14" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+    <row r="2" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-    </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+    </row>
+    <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -701,7 +736,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>5</v>
       </c>
@@ -717,7 +752,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B5" s="2"/>
       <c r="C5" s="2" t="s">
         <v>23</v>
@@ -731,7 +766,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:11" ht="30" x14ac:dyDescent="0.25">
       <c r="B6" s="2"/>
       <c r="C6" s="2" t="s">
         <v>25</v>
@@ -751,7 +786,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B7" s="3" t="s">
         <v>34</v>
       </c>
@@ -767,7 +802,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B8" s="3"/>
       <c r="C8" s="3" t="s">
         <v>21</v>
@@ -781,7 +816,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B9" s="3"/>
       <c r="C9" s="3" t="s">
         <v>20</v>
@@ -795,7 +830,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B10" s="3"/>
       <c r="C10" s="3" t="s">
         <v>19</v>
@@ -809,7 +844,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B11" s="3"/>
       <c r="C11" s="3" t="s">
         <v>18</v>
@@ -823,7 +858,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B12" s="3"/>
       <c r="C12" s="3" t="s">
         <v>29</v>
@@ -837,7 +872,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B13" s="3"/>
       <c r="C13" s="3" t="s">
         <v>13</v>
@@ -851,7 +886,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="14" spans="2:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:11" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="3"/>
       <c r="C14" s="3" t="s">
         <v>14</v>
@@ -865,7 +900,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="15" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B15" s="3"/>
       <c r="C15" s="3" t="s">
         <v>15</v>
@@ -879,7 +914,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B16" s="3"/>
       <c r="C16" s="3" t="s">
         <v>30</v>
@@ -892,8 +927,11 @@
         <f t="shared" si="0"/>
         <v>296</v>
       </c>
-    </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="K16" s="21" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
         <v>35</v>
       </c>
@@ -909,7 +947,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B18" s="3"/>
       <c r="C18" s="3" t="s">
         <v>31</v>
@@ -923,7 +961,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B19" s="3"/>
       <c r="C19" s="3" t="s">
         <v>33</v>
@@ -937,7 +975,7 @@
         <v>444</v>
       </c>
     </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B20" s="3"/>
       <c r="C20" s="3" t="s">
         <v>36</v>
@@ -951,7 +989,7 @@
         <v>592</v>
       </c>
     </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B21" s="3"/>
       <c r="C21" s="3" t="s">
         <v>37</v>
@@ -965,7 +1003,7 @@
         <v>296</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B22" s="3"/>
       <c r="C22" s="3" t="s">
         <v>38</v>
@@ -979,31 +1017,35 @@
         <v>148</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
+      <c r="C23" s="3" t="s">
+        <v>39</v>
+      </c>
       <c r="D23" s="2">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="24" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
+      <c r="C24" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="D24" s="2">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="10">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.25">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="25" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B25" s="4" t="s">
         <v>6</v>
       </c>
@@ -1019,7 +1061,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B26" s="5" t="s">
         <v>7</v>
       </c>
@@ -1035,7 +1077,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B27" s="5"/>
       <c r="C27" s="5" t="s">
         <v>12</v>
@@ -1049,7 +1091,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B28" s="8"/>
       <c r="C28" s="8" t="s">
         <v>28</v>
@@ -1062,8 +1104,9 @@
         <f>D28*$I$6</f>
         <v>370</v>
       </c>
-    </row>
-    <row r="29" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K28" s="19"/>
+    </row>
+    <row r="29" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6" t="s">
         <v>10</v>
       </c>
@@ -1077,22 +1120,28 @@
         <v>26</v>
       </c>
       <c r="I29" s="14">
-        <v>7600</v>
-      </c>
-    </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.25">
+        <v>8100</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="L29" s="18">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B30" s="9" t="s">
         <v>9</v>
       </c>
       <c r="C30" s="9"/>
       <c r="D30" s="9">
         <f>SUM(D4:D28)</f>
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="E30" s="9"/>
       <c r="F30" s="11">
         <f>SUM(F4:F29)</f>
-        <v>8808</v>
+        <v>10066</v>
       </c>
     </row>
     <row r="33" spans="8:9" x14ac:dyDescent="0.25">
@@ -1100,8 +1149,8 @@
         <v>27</v>
       </c>
       <c r="I33" s="16">
-        <f>F30-I29</f>
-        <v>1208</v>
+        <f>F30-I29-L29</f>
+        <v>1466</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se ha agregado un selector adicional para filtar por rango en la seción de filtrar por fechas
</commit_message>
<xml_diff>
--- a/Output/Precio de software TEKNOGADGET.xlsx
+++ b/Output/Precio de software TEKNOGADGET.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UZIEL\OneDrive\Documents\FREELANCER\TecnogadgedWin7\Output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6B98FE7-8208-4073-B6BD-00250C83D93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4631F5F-ACC6-4588-AE56-915F1CA2A346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{48C9FD5F-70C1-44D7-83C9-0F804B9CE7E4}"/>
+    <workbookView xWindow="4770" yWindow="555" windowWidth="21600" windowHeight="11295" xr2:uid="{48C9FD5F-70C1-44D7-83C9-0F804B9CE7E4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t>Modulos</t>
   </si>
@@ -163,6 +163,9 @@
   </si>
   <si>
     <t>15/3/2025 pago 700</t>
+  </si>
+  <si>
+    <t>Edición del registro de cliente, en estados "LABORATORIO" y "REPARADO"</t>
   </si>
 </sst>
 </file>
@@ -369,10 +372,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moneda" xfId="1" builtinId="4"/>
@@ -693,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE51DA6-4F34-4E63-B58F-F2E67A00BE67}">
-  <dimension ref="B2:L33"/>
+  <dimension ref="B2:L34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.42578125" customWidth="1"/>
@@ -711,13 +714,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="20"/>
-      <c r="D2" s="20"/>
-      <c r="E2" s="20"/>
-      <c r="F2" s="20"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
@@ -762,7 +765,7 @@
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="10">
-        <f t="shared" ref="F5:F24" si="0">D5*$I$6</f>
+        <f t="shared" ref="F5:F23" si="0">D5*$I$6</f>
         <v>74</v>
       </c>
     </row>
@@ -927,7 +930,7 @@
         <f t="shared" si="0"/>
         <v>296</v>
       </c>
-      <c r="K16" s="21" t="s">
+      <c r="K16" s="20" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1041,46 +1044,46 @@
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="10">
-        <f t="shared" si="0"/>
+        <f>D24*$I$6</f>
         <v>740</v>
       </c>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>16</v>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3" t="s">
+        <v>43</v>
       </c>
       <c r="D25" s="2">
-        <v>3</v>
-      </c>
-      <c r="E25" s="4"/>
+        <v>4</v>
+      </c>
+      <c r="E25" s="3"/>
       <c r="F25" s="10">
         <f>D25*$I$6</f>
-        <v>222</v>
+        <v>296</v>
       </c>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>11</v>
+      <c r="B26" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>16</v>
       </c>
       <c r="D26" s="2">
-        <v>2</v>
-      </c>
-      <c r="E26" s="5"/>
+        <v>3</v>
+      </c>
+      <c r="E26" s="4"/>
       <c r="F26" s="10">
         <f>D26*$I$6</f>
-        <v>148</v>
+        <v>222</v>
       </c>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="5"/>
+      <c r="B27" s="5" t="s">
+        <v>7</v>
+      </c>
       <c r="C27" s="5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D27" s="2">
         <v>2</v>
@@ -1091,66 +1094,80 @@
         <v>148</v>
       </c>
     </row>
-    <row r="28" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="8"/>
-      <c r="C28" s="8" t="s">
-        <v>28</v>
+    <row r="28" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="5"/>
+      <c r="C28" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="D28" s="2">
-        <v>5</v>
-      </c>
-      <c r="E28" s="8"/>
+        <v>2</v>
+      </c>
+      <c r="E28" s="5"/>
       <c r="F28" s="10">
         <f>D28*$I$6</f>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="29" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="8"/>
+      <c r="C29" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="D29" s="2">
+        <v>5</v>
+      </c>
+      <c r="E29" s="8"/>
+      <c r="F29" s="10">
+        <f>D29*$I$6</f>
         <v>370</v>
       </c>
-      <c r="K28" s="19"/>
-    </row>
-    <row r="29" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="6" t="s">
+      <c r="K29" s="19"/>
+    </row>
+    <row r="30" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C29" s="6"/>
-      <c r="D29" s="6"/>
-      <c r="E29" s="6"/>
-      <c r="F29" s="10">
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="10">
         <v>2000</v>
       </c>
-      <c r="H29" s="13" t="s">
+      <c r="H30" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="I29" s="14">
-        <v>8100</v>
-      </c>
-      <c r="K29" s="17" t="s">
+      <c r="I30" s="14">
+        <v>8800</v>
+      </c>
+      <c r="K30" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="L29" s="18">
+      <c r="L30" s="18">
         <v>500</v>
       </c>
     </row>
-    <row r="30" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B30" s="9" t="s">
+    <row r="31" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B31" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C30" s="9"/>
-      <c r="D30" s="9">
-        <f>SUM(D4:D28)</f>
-        <v>109</v>
-      </c>
-      <c r="E30" s="9"/>
-      <c r="F30" s="11">
-        <f>SUM(F4:F29)</f>
-        <v>10066</v>
-      </c>
-    </row>
-    <row r="33" spans="8:9" x14ac:dyDescent="0.25">
-      <c r="H33" s="15" t="s">
+      <c r="C31" s="9"/>
+      <c r="D31" s="9">
+        <f>SUM(D4:D29)</f>
+        <v>113</v>
+      </c>
+      <c r="E31" s="9"/>
+      <c r="F31" s="11">
+        <f>SUM(F4:F30)</f>
+        <v>10362</v>
+      </c>
+    </row>
+    <row r="34" spans="8:9" x14ac:dyDescent="0.25">
+      <c r="H34" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="I33" s="16">
-        <f>F30-I29-L29</f>
-        <v>1466</v>
+      <c r="I34" s="16">
+        <f>F31-I30-L30</f>
+        <v>1062</v>
       </c>
     </row>
   </sheetData>

</xml_diff>